<commit_message>
[WEB OPR JMTO] - memperbaharui template import petugas, membuat function getJabatanId
</commit_message>
<xml_diff>
--- a/public/assets/template/template_import_petugas.xlsx
+++ b/public/assets/template/template_import_petugas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c38e22937a30378c/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haidarijlal\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="8_{2CCA4049-CDD7-4C30-9524-779103D419A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17EAA838-9F30-45E8-AEEF-03D9BEDC1F4F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69DDBD9C-2BCE-460D-855D-B456C389EDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{5ED6FD84-7A7E-4234-BAA8-B266A2729A67}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>NPP PETUGAS</t>
   </si>
@@ -42,22 +42,13 @@
     <t>NAMA PETUGAS</t>
   </si>
   <si>
-    <t>Haidar</t>
-  </si>
-  <si>
     <t>EMAIL</t>
-  </si>
-  <si>
-    <t>user@user.com</t>
   </si>
   <si>
     <t>PASSWORD</t>
   </si>
   <si>
-    <t>user2@user.com</t>
-  </si>
-  <si>
-    <t>ijlal</t>
+    <t>JABATAN</t>
   </si>
 </sst>
 </file>
@@ -433,10 +424,10 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.35">
@@ -444,50 +435,31 @@
         <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" s="1"/>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B3">
-        <v>10102</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3">
-        <v>10102</v>
-      </c>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B4">
-        <v>10101</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E4">
-        <v>10101</v>
-      </c>
+      <c r="C4" s="2"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" xr:uid="{D7F1770D-E179-4723-8E86-36C77A09A670}"/>
-    <hyperlink ref="C3" r:id="rId2" xr:uid="{3861D56F-7DB1-45A0-B70F-53971F37179D}"/>
-  </hyperlinks>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D1048576" xr:uid="{4868F774-ADD9-4783-95CE-2120F5697628}">
+      <formula1>"KBT,KSPT,PLT,TEKNISI"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[WEB OPR JMTO] - Merubah filled data yang di import
</commit_message>
<xml_diff>
--- a/public/assets/template/template_import_petugas.xlsx
+++ b/public/assets/template/template_import_petugas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haidarijlal\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\www\Jasa Marga Tollroad Operator\operasional_jmto\public\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69DDBD9C-2BCE-460D-855D-B456C389EDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7880F8BA-70CC-448D-93D3-FE5155B10470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{5ED6FD84-7A7E-4234-BAA8-B266A2729A67}"/>
+    <workbookView xWindow="30450" yWindow="1650" windowWidth="21600" windowHeight="11715" xr2:uid="{5ED6FD84-7A7E-4234-BAA8-B266A2729A67}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,13 +42,13 @@
     <t>NAMA PETUGAS</t>
   </si>
   <si>
-    <t>EMAIL</t>
+    <t>JABATAN</t>
   </si>
   <si>
-    <t>PASSWORD</t>
+    <t>KSPT</t>
   </si>
   <si>
-    <t>JABATAN</t>
+    <t>haidar ijlal</t>
   </si>
 </sst>
 </file>
@@ -420,17 +420,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E87C21E8-984A-4862-8C9A-625F9A499FC8}">
-  <dimension ref="B2:F4"/>
+  <dimension ref="B2:E4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -438,24 +438,27 @@
         <v>2</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B3">
+        <v>210600</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>3</v>
-      </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
       <c r="C4" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D1048576" xr:uid="{4868F774-ADD9-4783-95CE-2120F5697628}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1 C3:C1048576" xr:uid="{4868F774-ADD9-4783-95CE-2120F5697628}">
       <formula1>"KBT,KSPT,PLT,TEKNISI"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
[WEB OPR JMTO] - Memperbaiki bugs empty row in excel
</commit_message>
<xml_diff>
--- a/public/assets/template/template_import_petugas.xlsx
+++ b/public/assets/template/template_import_petugas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\www\Jasa Marga Tollroad Operator\operasional_jmto\public\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7880F8BA-70CC-448D-93D3-FE5155B10470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB6AB0A6-46BE-44B0-9F2A-2CFDEED9CA73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30450" yWindow="1650" windowWidth="21600" windowHeight="11715" xr2:uid="{5ED6FD84-7A7E-4234-BAA8-B266A2729A67}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{EC9E512E-EC17-48F2-93A2-6B3679A2BE84}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,28 +34,22 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>NPP PETUGAS</t>
-  </si>
-  <si>
-    <t>NAMA PETUGAS</t>
   </si>
   <si>
     <t>JABATAN</t>
   </si>
   <si>
-    <t>KSPT</t>
-  </si>
-  <si>
-    <t>haidar ijlal</t>
+    <t>NAMA PETUGAS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -67,14 +61,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -97,17 +83,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -419,50 +402,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E87C21E8-984A-4862-8C9A-625F9A499FC8}">
-  <dimension ref="B2:E4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50C6E759-E983-4A76-A9A7-E6123A49C2DF}">
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B2" s="1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B3">
-        <v>210600</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="C4" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1 C3:C1048576" xr:uid="{4868F774-ADD9-4783-95CE-2120F5697628}">
-      <formula1>"KBT,KSPT,PLT,TEKNISI"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{71EC0A47-B816-4C01-BAF5-9F4E5BEC8B96}">
+      <formula1>"KSPT,KBT,PLT,TEKNISI"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>